<commit_message>
[Nairne] Sync armada-innovations-2026.xlsx with brokerage attribution + sweep timing
- New Brokerage Attribution tab matching the standalone xlsx (Mar 31 → Apr → May 2 flow)
- Capital Roll: added note explaining why Net Ending Capital is $0 each month
  (GP sweeps distribution out at start of next month)
- Source Trail: added two GP-rule rows documenting the sweep timing for Mar
  (paid out Apr 1) and Apr (still in brokerage, sweeps May 1+)
- Member Distribution: added ITD Member Earnings summary at the bottom
  (Nairne $73,983.74 / Alec $48,705.96 / Chris $616.53 = $123,306.23)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/armada-innovations/data/armada-innovations-2026.xlsx
+++ b/armada-innovations/data/armada-innovations-2026.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capital Roll" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fund Source" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Trail" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brokerage Attribution" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00;[Red](&quot;$&quot;#,##0.00)"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +59,25 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="004A5568"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -76,8 +94,33 @@
         <fgColor rgb="002A3550"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE9FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -99,11 +142,69 @@
         <color rgb="00888888"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00888888"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00888888"/>
+      </right>
+      <top style="thin">
+        <color rgb="00888888"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00888888"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00888888"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00888888"/>
+      </right>
+      <top style="thin">
+        <color rgb="00888888"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00888888"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -133,6 +234,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -996,7 +1125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1352,37 +1481,30 @@
       <c r="G15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Alec Atkinson</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="8" t="n">
-        <v>0.395</v>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Capital Relations</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Armada Innovations LLC</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr"/>
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>ITD Member Earnings (Mar+Apr 2026)</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="n"/>
+      <c r="C16" s="22" t="n"/>
+      <c r="D16" s="22" t="n"/>
+      <c r="E16" s="22" t="n"/>
+      <c r="F16" s="22" t="n"/>
+      <c r="G16" s="23" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Chris (TBD last name)</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="8" t="n">
-        <v>0.005</v>
+          <t>Nairne (60%)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>73983.74000000001</v>
+      </c>
+      <c r="C17" s="8">
+        <f> $2,232.00 (Mar) + $71,751.74 (Apr)</f>
+        <v/>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
@@ -1404,12 +1526,14 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Total Share</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr"/>
+          <t>Alec (39.5%)</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>48705.96</v>
+      </c>
       <c r="C18" s="9">
-        <f>SUM(C11:C13)</f>
+        <f> $1,469.40 (Mar) + $47,236.56 (Apr)</f>
         <v/>
       </c>
       <c r="D18" s="6" t="inlineStr"/>
@@ -1421,8 +1545,34 @@
       </c>
       <c r="G18" s="6" t="inlineStr"/>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Chris (0.5%)</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n">
+        <v>616.53</v>
+      </c>
+      <c r="C19">
+        <f> $18.60 (Mar) + $597.93 (Apr)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>Total ITD</t>
+        </is>
+      </c>
+      <c r="B20" s="25">
+        <f>B17+B18+B19</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1435,7 +1585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1664,9 +1814,25 @@
         <v>0</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>Note: GP sweep timing</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>Innovations LLC sweeps its monthly distribution out of the fund at the start of the next month. Net Ending Capital is $0 each month because the distribution clears the account.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="A15:E15"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2042,7 +2208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2344,10 +2510,350 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>GP rule</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>Sweep timing — Innovations LLC</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>GP distribution swept from brokerage to Innovations bank at the start of the next month</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>Mar $3,720 swept Apr 1 → Nairne $2,232 / Alec $1,469.40 / Chris $18.60 (already paid out)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>GP rule</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>April distribution status</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>Apr GP $119,586.23 still in brokerage as of May 2, awaiting May 1+ sweep</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>Will pay out: Nairne $71,751.74 / Alec $47,236.56 / Chris $597.93</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Armada Capital Group LLP — Brokerage Attribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>As of May 2, 2026 · Brokerage value $10,519,780</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>GP rule: Innovations LLC sweeps its monthly distribution at the start of the next month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Mar GP $3,720 swept Apr 1 (Innovations had $0 in fund during April).  Apr GP $119,586.23 sits in brokerage today, sweeps at start of May.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>Capital Contributed</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>Mar 31 Bal
+(= Apr 1 Beg)</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>+ Apr Activity
+(net of fees)</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="inlineStr">
+        <is>
+          <t>+ May Wire
+(advance)</t>
+        </is>
+      </c>
+      <c r="F6" s="29" t="inlineStr">
+        <is>
+          <t>Current Balance
+(May 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>Bliss Investments LLC</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="n">
+        <v>500000</v>
+      </c>
+      <c r="C7" s="31" t="n">
+        <v>508472</v>
+      </c>
+      <c r="D7" s="31" t="n">
+        <v>16636.19</v>
+      </c>
+      <c r="E7" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="31" t="n">
+        <v>525108.1899999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>JJNA, LLC</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="C8" s="31" t="n">
+        <v>8020000</v>
+      </c>
+      <c r="D8" s="31" t="n">
+        <v>262398.36</v>
+      </c>
+      <c r="E8" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="31" t="n">
+        <v>8282398.36</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="32" t="inlineStr">
+        <is>
+          <t>New May Investors</t>
+        </is>
+      </c>
+      <c r="B9" s="33" t="n">
+        <v>1499728</v>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="33" t="n">
+        <v>1499728</v>
+      </c>
+      <c r="F9" s="33" t="n">
+        <v>1499728</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>TruQuant (accrued payable)</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="35" t="n">
+        <v>87502.12</v>
+      </c>
+      <c r="E10" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="35" t="n">
+        <v>87502.12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="36" t="inlineStr">
+        <is>
+          <t>Innovations GP (Apr accrual, awaiting May sweep)</t>
+        </is>
+      </c>
+      <c r="B11" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="37" t="n">
+        <v>119586.23</v>
+      </c>
+      <c r="E11" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="37" t="n">
+        <v>119586.23</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="38" t="inlineStr">
+        <is>
+          <t>Bank-fee cash carry</t>
+        </is>
+      </c>
+      <c r="B12" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="39" t="n">
+        <v>-135.9</v>
+      </c>
+      <c r="D12" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="39" t="n">
+        <v>-135.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>TOTAL ATTRIBUTED</t>
+        </is>
+      </c>
+      <c r="B13" s="41">
+        <f>SUM(B7:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="41">
+        <f>SUM(C7:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="41">
+        <f>SUM(D7:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="41">
+        <f>SUM(E7:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="41">
+        <f>SUM(F7:F12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="42" t="inlineStr">
+        <is>
+          <t>Brokerage actual (live)</t>
+        </is>
+      </c>
+      <c r="B14" s="43" t="n"/>
+      <c r="C14" s="43" t="n"/>
+      <c r="D14" s="43" t="n"/>
+      <c r="E14" s="43" t="n"/>
+      <c r="F14" s="44" t="n">
+        <v>10519780</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="42" t="inlineStr">
+        <is>
+          <t>LEFTOVER (≈3 days fund growth)</t>
+        </is>
+      </c>
+      <c r="B15" s="43" t="n"/>
+      <c r="C15" s="43" t="n"/>
+      <c r="D15" s="43" t="n"/>
+      <c r="E15" s="43" t="n"/>
+      <c r="F15" s="44">
+        <f>F14-F13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>Already paid out (not in current brokerage):</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Mar 2026 GP distribution $3,720 swept Apr 1 to Innovations bank — Nairne $2,232.00 / Alec $1,469.40 / Chris $18.60</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A3:F3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
[Nairne] Add Monthly Profit Breakdown tab — full waterfall by month
New tab (placed first in workbook) showing complete monthly profit
breakdown side-by-side for Mar and Apr 2026, plus ITD Total:

- Inputs: LP beginning balances per month
- Gross fund profit
- Waterfall:
  • TruQuant (Traders): 18% of gross
  • LPs: 57.4% of gross, pro-rata by LP balance (Bliss + JJNA)
  • GP / Innovations LLC: 24.6%, split Nairne 60% / Alec 39.5% / Chris 0.5%
- Verification row (sums must = gross)
- Expenses + Net income
- Reference notes including March exception (realized→GP / unrealized→LP)
  and GP monthly sweep timing

Every recipient shows their $ amount AND % of gross / % of their slice.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/armada-innovations/data/armada-innovations-2026.xlsx
+++ b/armada-innovations/data/armada-innovations-2026.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Level" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Member Distribution" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capital Roll" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fund Source" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Trail" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brokerage Attribution" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Profit Breakdown" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Level" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Member Distribution" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capital Roll" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fund Source" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Trail" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brokerage Attribution" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,8 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00;[Red](&quot;$&quot;#,##0.00)"/>
+    <numFmt numFmtId="165" formatCode="0.000%"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -204,7 +206,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -262,6 +264,29 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="9" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="9" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="9" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="9" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="9" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -627,6 +652,790 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Monthly Profit Breakdown — Total Profits &amp; Who Gets What</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Armada Capital Group LLP · Mar–Apr 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="inlineStr">
+        <is>
+          <t>Recipient</t>
+        </is>
+      </c>
+      <c r="C4" s="29" t="inlineStr">
+        <is>
+          <t>% of Gross</t>
+        </is>
+      </c>
+      <c r="D4" s="29" t="inlineStr">
+        <is>
+          <t>March 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="29" t="inlineStr">
+        <is>
+          <t>% of Mar</t>
+        </is>
+      </c>
+      <c r="F4" s="29" t="inlineStr">
+        <is>
+          <t>April 2026</t>
+        </is>
+      </c>
+      <c r="G4" s="29" t="inlineStr">
+        <is>
+          <t>% of Apr</t>
+        </is>
+      </c>
+      <c r="H4" s="29" t="inlineStr">
+        <is>
+          <t>ITD Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="45" t="inlineStr">
+        <is>
+          <t>INPUTS — Beginning LP Capital (= base for waterfall)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Bliss Investments LLC</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
+      <c r="C6" s="46" t="n"/>
+      <c r="D6" s="31" t="n">
+        <v>508472</v>
+      </c>
+      <c r="E6" s="46" t="n"/>
+      <c r="F6" s="31" t="n">
+        <v>508472</v>
+      </c>
+      <c r="G6" s="46" t="n"/>
+      <c r="H6" s="31" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  JJNA, LLC</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
+      <c r="C7" s="46" t="n"/>
+      <c r="D7" s="31" t="n">
+        <v>8020000</v>
+      </c>
+      <c r="E7" s="46" t="n"/>
+      <c r="F7" s="31" t="n">
+        <v>8020000</v>
+      </c>
+      <c r="G7" s="46" t="n"/>
+      <c r="H7" s="31" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total LP Base</t>
+        </is>
+      </c>
+      <c r="B8" s="42" t="inlineStr"/>
+      <c r="C8" s="42" t="n"/>
+      <c r="D8" s="44" t="n">
+        <v>8528472</v>
+      </c>
+      <c r="E8" s="42" t="n"/>
+      <c r="F8" s="44" t="n">
+        <v>8528472</v>
+      </c>
+      <c r="G8" s="42" t="n"/>
+      <c r="H8" s="44" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="45" t="inlineStr">
+        <is>
+          <t>GROSS FUND PROFIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Gross profit for the month</t>
+        </is>
+      </c>
+      <c r="B11" s="42" t="inlineStr"/>
+      <c r="C11" s="42" t="n"/>
+      <c r="D11" s="44" t="n">
+        <v>32400</v>
+      </c>
+      <c r="E11" s="42" t="n"/>
+      <c r="F11" s="44" t="n">
+        <v>486122.9</v>
+      </c>
+      <c r="G11" s="42" t="n"/>
+      <c r="H11" s="44" t="n">
+        <v>518522.9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Effective % return on LP base</t>
+        </is>
+      </c>
+      <c r="B12" s="43" t="inlineStr"/>
+      <c r="C12" s="43" t="n"/>
+      <c r="D12" s="39" t="n"/>
+      <c r="E12" s="47" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="F12" s="39" t="n"/>
+      <c r="G12" s="47" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="H12" s="39" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="45" t="inlineStr">
+        <is>
+          <t>WATERFALL — TruQuant (Traders)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TruQuant performance fee</t>
+        </is>
+      </c>
+      <c r="B15" s="34" t="inlineStr">
+        <is>
+          <t>Traders</t>
+        </is>
+      </c>
+      <c r="C15" s="48" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D15" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="49" t="n">
+        <v>87502.12</v>
+      </c>
+      <c r="G15" s="50" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H15" s="49" t="n">
+        <v>87502.12</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Note: March had no TQ fee</t>
+        </is>
+      </c>
+      <c r="B16" s="43" t="inlineStr"/>
+      <c r="C16" s="43" t="n"/>
+      <c r="D16" s="39" t="n"/>
+      <c r="E16" s="43" t="n"/>
+      <c r="F16" s="39" t="n"/>
+      <c r="G16" s="43" t="n"/>
+      <c r="H16" s="39" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="45" t="inlineStr">
+        <is>
+          <t>WATERFALL — Armada Capital Group (82% of gross)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ACG Total</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t>Fund</t>
+        </is>
+      </c>
+      <c r="C19" s="52" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D19" s="44" t="n">
+        <v>32400</v>
+      </c>
+      <c r="E19" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="44" t="n">
+        <v>398620.78</v>
+      </c>
+      <c r="G19" s="53" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="H19" s="44" t="n">
+        <v>431020.78</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    LPs (70% of ACG = 57.4% of gross)</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>LP slice</t>
+        </is>
+      </c>
+      <c r="C20" s="54" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="D20" s="55" t="n">
+        <v>28680</v>
+      </c>
+      <c r="E20" s="56" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="F20" s="55" t="n">
+        <v>279034.55</v>
+      </c>
+      <c r="G20" s="56" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="H20" s="55" t="n">
+        <v>307714.55</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Bliss Investments LLC</t>
+        </is>
+      </c>
+      <c r="B21" s="46" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
+      <c r="C21" s="46" t="n"/>
+      <c r="D21" s="31" t="n">
+        <v>8680</v>
+      </c>
+      <c r="E21" s="57" t="n">
+        <v>0.302649930264993</v>
+      </c>
+      <c r="F21" s="31" t="n">
+        <v>16636.19</v>
+      </c>
+      <c r="G21" s="57" t="n">
+        <v>0.05962053803014716</v>
+      </c>
+      <c r="H21" s="31" t="n">
+        <v>25316.19</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      JJNA, LLC</t>
+        </is>
+      </c>
+      <c r="B22" s="46" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
+      <c r="C22" s="46" t="n"/>
+      <c r="D22" s="31" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E22" s="57" t="n">
+        <v>0.697350069735007</v>
+      </c>
+      <c r="F22" s="31" t="n">
+        <v>262398.36</v>
+      </c>
+      <c r="G22" s="57" t="n">
+        <v>0.9403794619698528</v>
+      </c>
+      <c r="H22" s="31" t="n">
+        <v>282398.36</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    GP / Innovations LLC (30% of ACG = 24.6% of gross)</t>
+        </is>
+      </c>
+      <c r="B23" s="36" t="inlineStr">
+        <is>
+          <t>GP slice</t>
+        </is>
+      </c>
+      <c r="C23" s="58" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="D23" s="59" t="n">
+        <v>3720</v>
+      </c>
+      <c r="E23" s="60" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="F23" s="59" t="n">
+        <v>119586.23</v>
+      </c>
+      <c r="G23" s="60" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="H23" s="59" t="n">
+        <v>123306.23</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Nairne (60% of GP slice)</t>
+        </is>
+      </c>
+      <c r="B24" s="61" t="inlineStr">
+        <is>
+          <t>GP</t>
+        </is>
+      </c>
+      <c r="C24" s="61" t="n"/>
+      <c r="D24" s="37" t="n">
+        <v>2232</v>
+      </c>
+      <c r="E24" s="62" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F24" s="37" t="n">
+        <v>71751.74000000001</v>
+      </c>
+      <c r="G24" s="62" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H24" s="37" t="n">
+        <v>73983.74000000001</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Alec (39.5% of GP slice)</t>
+        </is>
+      </c>
+      <c r="B25" s="61" t="inlineStr">
+        <is>
+          <t>GP</t>
+        </is>
+      </c>
+      <c r="C25" s="61" t="n"/>
+      <c r="D25" s="37" t="n">
+        <v>1469.4</v>
+      </c>
+      <c r="E25" s="62" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="F25" s="37" t="n">
+        <v>47236.56</v>
+      </c>
+      <c r="G25" s="62" t="n">
+        <v>0.395</v>
+      </c>
+      <c r="H25" s="37" t="n">
+        <v>48705.96</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Chris (0.5% of GP slice)</t>
+        </is>
+      </c>
+      <c r="B26" s="61" t="inlineStr">
+        <is>
+          <t>GP</t>
+        </is>
+      </c>
+      <c r="C26" s="61" t="n"/>
+      <c r="D26" s="37" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="E26" s="62" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="F26" s="37" t="n">
+        <v>597.9299999999999</v>
+      </c>
+      <c r="G26" s="62" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="H26" s="37" t="n">
+        <v>616.53</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="45" t="inlineStr">
+        <is>
+          <t>VERIFICATION — must equal Gross Profit</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sum of all distributions</t>
+        </is>
+      </c>
+      <c r="B29" s="63" t="n"/>
+      <c r="C29" s="63" t="n"/>
+      <c r="D29" s="44" t="n">
+        <v>32400</v>
+      </c>
+      <c r="E29" s="63" t="n"/>
+      <c r="F29" s="44" t="n">
+        <v>486122.9</v>
+      </c>
+      <c r="G29" s="63" t="n"/>
+      <c r="H29" s="44" t="n">
+        <v>518522.9</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Gross profit (above)</t>
+        </is>
+      </c>
+      <c r="B30" s="43" t="n"/>
+      <c r="C30" s="43" t="n"/>
+      <c r="D30" s="39" t="n">
+        <v>32400</v>
+      </c>
+      <c r="E30" s="43" t="n"/>
+      <c r="F30" s="39" t="n">
+        <v>486122.9</v>
+      </c>
+      <c r="G30" s="43" t="n"/>
+      <c r="H30" s="39" t="n">
+        <v>518522.9</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tie-out (must = $0)</t>
+        </is>
+      </c>
+      <c r="B31" s="63" t="n"/>
+      <c r="C31" s="63" t="n"/>
+      <c r="D31" s="64">
+        <f>D29-D30</f>
+        <v/>
+      </c>
+      <c r="E31" s="63" t="n"/>
+      <c r="F31" s="64">
+        <f>F29-F30</f>
+        <v/>
+      </c>
+      <c r="G31" s="63" t="n"/>
+      <c r="H31" s="64">
+        <f>H29-H30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="45" t="inlineStr">
+        <is>
+          <t>FUND EXPENSES (TPA-level, separate from waterfall)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Bank fees</t>
+        </is>
+      </c>
+      <c r="B34" s="65" t="inlineStr"/>
+      <c r="C34" s="63" t="n"/>
+      <c r="D34" s="64" t="n">
+        <v>180.9</v>
+      </c>
+      <c r="E34" s="63" t="n"/>
+      <c r="F34" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="63" t="n"/>
+      <c r="H34" s="64" t="n">
+        <v>180.9</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Note: Apr bank fees not yet booked (preliminary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="45" t="inlineStr">
+        <is>
+          <t>NET INCOME / LOSS (Income Statement basis, sign-flipped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total revenue</t>
+        </is>
+      </c>
+      <c r="B37" s="63" t="inlineStr"/>
+      <c r="C37" s="63" t="n"/>
+      <c r="D37" s="64" t="n">
+        <v>-32400</v>
+      </c>
+      <c r="E37" s="63" t="n"/>
+      <c r="F37" s="64" t="n">
+        <v>-486122.9</v>
+      </c>
+      <c r="G37" s="63" t="n"/>
+      <c r="H37" s="64" t="n">
+        <v>-518522.9</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total expense</t>
+        </is>
+      </c>
+      <c r="B38" s="63" t="inlineStr"/>
+      <c r="C38" s="63" t="n"/>
+      <c r="D38" s="64" t="n">
+        <v>180.9</v>
+      </c>
+      <c r="E38" s="63" t="n"/>
+      <c r="F38" s="64" t="n">
+        <v>87502.12</v>
+      </c>
+      <c r="G38" s="63" t="n"/>
+      <c r="H38" s="64" t="n">
+        <v>87683.02</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Net income (loss)</t>
+        </is>
+      </c>
+      <c r="B39" s="42" t="inlineStr"/>
+      <c r="C39" s="42" t="n"/>
+      <c r="D39" s="44" t="n">
+        <v>-32219.1</v>
+      </c>
+      <c r="E39" s="42" t="n"/>
+      <c r="F39" s="44" t="n">
+        <v>-398620.78</v>
+      </c>
+      <c r="G39" s="42" t="n"/>
+      <c r="H39" s="44" t="n">
+        <v>-430839.88</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="45" t="inlineStr">
+        <is>
+          <t>REFERENCE — Waterfall Logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="26" t="inlineStr">
+        <is>
+          <t>Standard waterfall (April onward):</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  18% to TruQuant (traders) straight off the top</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  82% to Armada Capital Group LLP, split:</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    70% of ACG slice (= 57.4% of gross) to LPs, pro-rata by beginning balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    30% of ACG slice (= 24.6% of gross) to Innovations LLC (GP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="26" t="inlineStr">
+        <is>
+          <t>Innovations LLC member split:</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Nairne 60% / Alec 39.5% / Chris 0.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="26" t="inlineStr">
+        <is>
+          <t>GP sweep timing:</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Innovations LLC sweeps its monthly distribution at the start of the next month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Mar GP $3,720 swept Apr 1 (during April Innovations had $0 in fund).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Apr GP $119,586.23 sits in brokerage today, sweeps at start of May.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="26" t="inlineStr">
+        <is>
+          <t>March exception:</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  March allocation followed PE/RE template (realized gains 100% to GP, unrealized 100% to LPs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  No TruQuant fee accrued in March.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="24">
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A54:H54"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A53:H53"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A44:H44"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1119,7 +1928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1579,7 +2388,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1838,7 +2647,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2202,7 +3011,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2562,7 +3371,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>